<commit_message>
Updated for processed values
</commit_message>
<xml_diff>
--- a/static/fields/researchcovidmirnaandproteomics_reference.xlsx
+++ b/static/fields/researchcovidmirnaandproteomics_reference.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/violet.wren/WebstormProjects/open.fda.gov/static/fields/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7B1106CF-29A1-0F4F-9676-74CFBAE9FD30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76732E2F-8D8B-4C45-BBBC-818C862C3B61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="21900" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="40">
   <si>
     <t>Field Name</t>
   </si>
@@ -81,9 +81,6 @@
     <t>Name of the measured control</t>
   </si>
   <si>
-    <t>Value of the measured control</t>
-  </si>
-  <si>
     <t>housekeeping_gene_controls</t>
   </si>
   <si>
@@ -105,9 +102,6 @@
     <t>Name of the measured miRNA</t>
   </si>
   <si>
-    <t>Value of the measured miRNA</t>
-  </si>
-  <si>
     <t>Value of the measured protein</t>
   </si>
   <si>
@@ -136,6 +130,21 @@
   </si>
   <si>
     <t>Unique sample IDs</t>
+  </si>
+  <si>
+    <t>processed_value</t>
+  </si>
+  <si>
+    <t>raw_value</t>
+  </si>
+  <si>
+    <t>Processed value of the measured control</t>
+  </si>
+  <si>
+    <t>Raw value of the measured control</t>
+  </si>
+  <si>
+    <t>double</t>
   </si>
 </sst>
 </file>
@@ -998,7 +1007,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D751"/>
+  <dimension ref="A1:D754"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.1640625" style="3" bestFit="1" customWidth="1"/>
@@ -1030,7 +1039,7 @@
         <v>4</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="34" x14ac:dyDescent="0.2">
@@ -1041,7 +1050,7 @@
         <v>4</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -1052,7 +1061,7 @@
         <v>4</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -1063,7 +1072,7 @@
         <v>6</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -1075,7 +1084,7 @@
         <v>4</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="17" x14ac:dyDescent="0.2">
@@ -1087,7 +1096,7 @@
         <v>4</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
@@ -1118,162 +1127,195 @@
         <v>13</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D10" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A11" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" s="4"/>
+      <c r="B12" s="4" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="4"/>
-      <c r="B11" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C11" s="3" t="s">
+      <c r="C12" s="3" t="s">
         <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A12" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C13" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A14" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D13" s="5" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="4"/>
-      <c r="B14" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>14</v>
+      <c r="D14" s="5" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B15" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" s="4"/>
+      <c r="B16" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A17" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C17" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D15" s="5" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="17" x14ac:dyDescent="0.2">
-      <c r="A16" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="4"/>
-      <c r="B17" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>14</v>
+      <c r="D17" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="4" t="s">
-        <v>21</v>
-      </c>
+        <v>37</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A20" s="4"/>
       <c r="B20" s="4" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="17" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="C21" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A22" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="17" x14ac:dyDescent="0.2">
+      <c r="A24" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B24" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C24" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D21" s="5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" s="4"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="4"/>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="4"/>
+      <c r="D24" s="5" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" s="4"/>
@@ -1368,16 +1410,16 @@
     <row r="55" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A55" s="4"/>
     </row>
-    <row r="56" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A56" s="4"/>
+    </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A57" s="4"/>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A58" s="4"/>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A59" s="4"/>
-    </row>
+    <row r="59" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="60" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A60" s="4"/>
     </row>
@@ -1402,16 +1444,16 @@
     <row r="67" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A67" s="4"/>
     </row>
-    <row r="68" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A68" s="4"/>
+    </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A69" s="4"/>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A70" s="4"/>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A71" s="4"/>
-    </row>
+    <row r="71" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="72" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A72" s="4"/>
     </row>
@@ -1508,16 +1550,16 @@
     <row r="103" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A103" s="4"/>
     </row>
-    <row r="104" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="104" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A104" s="4"/>
+    </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A105" s="4"/>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A106" s="4"/>
     </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A107" s="4"/>
-    </row>
+    <row r="107" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="108" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A108" s="4"/>
     </row>
@@ -1542,16 +1584,16 @@
     <row r="115" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A115" s="4"/>
     </row>
-    <row r="116" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="116" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A116" s="4"/>
+    </row>
     <row r="117" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A117" s="4"/>
     </row>
     <row r="118" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A118" s="4"/>
     </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A119" s="4"/>
-    </row>
+    <row r="119" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="120" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A120" s="4"/>
     </row>
@@ -1648,16 +1690,16 @@
     <row r="151" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A151" s="4"/>
     </row>
-    <row r="158" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="159" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A159" s="4"/>
-    </row>
-    <row r="160" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A160" s="4"/>
-    </row>
-    <row r="161" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A161" s="4"/>
-    </row>
+    <row r="152" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A152" s="4"/>
+    </row>
+    <row r="153" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A153" s="4"/>
+    </row>
+    <row r="154" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A154" s="4"/>
+    </row>
+    <row r="161" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="162" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A162" s="4"/>
     </row>
@@ -1682,16 +1724,16 @@
     <row r="169" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A169" s="4"/>
     </row>
-    <row r="170" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="170" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A170" s="4"/>
+    </row>
     <row r="171" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A171" s="4"/>
     </row>
     <row r="172" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A172" s="4"/>
     </row>
-    <row r="173" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A173" s="4"/>
-    </row>
+    <row r="173" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="174" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A174" s="4"/>
     </row>
@@ -1716,15 +1758,15 @@
     <row r="181" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A181" s="4"/>
     </row>
+    <row r="182" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A182" s="4"/>
+    </row>
     <row r="183" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A183" s="4"/>
     </row>
     <row r="184" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A184" s="4"/>
     </row>
-    <row r="185" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A185" s="4"/>
-    </row>
     <row r="186" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A186" s="4"/>
     </row>
@@ -1749,15 +1791,15 @@
     <row r="193" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A193" s="4"/>
     </row>
+    <row r="194" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A194" s="4"/>
+    </row>
     <row r="195" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A195" s="4"/>
     </row>
     <row r="196" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A196" s="4"/>
     </row>
-    <row r="197" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A197" s="4"/>
-    </row>
     <row r="198" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A198" s="4"/>
     </row>
@@ -1782,16 +1824,16 @@
     <row r="205" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A205" s="4"/>
     </row>
-    <row r="206" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="206" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A206" s="4"/>
+    </row>
     <row r="207" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A207" s="4"/>
     </row>
     <row r="208" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A208" s="4"/>
     </row>
-    <row r="209" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A209" s="4"/>
-    </row>
+    <row r="209" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="210" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A210" s="4"/>
     </row>
@@ -1816,16 +1858,16 @@
     <row r="217" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A217" s="4"/>
     </row>
-    <row r="218" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="218" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A218" s="4"/>
+    </row>
     <row r="219" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A219" s="4"/>
     </row>
     <row r="220" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A220" s="4"/>
     </row>
-    <row r="221" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A221" s="4"/>
-    </row>
+    <row r="221" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="222" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A222" s="4"/>
     </row>
@@ -1850,15 +1892,15 @@
     <row r="229" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A229" s="4"/>
     </row>
+    <row r="230" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A230" s="4"/>
+    </row>
     <row r="231" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A231" s="4"/>
     </row>
     <row r="232" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A232" s="4"/>
     </row>
-    <row r="233" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A233" s="4"/>
-    </row>
     <row r="234" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A234" s="4"/>
     </row>
@@ -1883,15 +1925,15 @@
     <row r="241" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A241" s="4"/>
     </row>
+    <row r="242" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A242" s="4"/>
+    </row>
     <row r="243" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A243" s="4"/>
     </row>
     <row r="244" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A244" s="4"/>
     </row>
-    <row r="245" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A245" s="4"/>
-    </row>
     <row r="246" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A246" s="4"/>
     </row>
@@ -1916,16 +1958,16 @@
     <row r="253" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A253" s="4"/>
     </row>
-    <row r="254" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="254" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A254" s="4"/>
+    </row>
     <row r="255" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A255" s="4"/>
     </row>
     <row r="256" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A256" s="4"/>
     </row>
-    <row r="257" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A257" s="4"/>
-    </row>
+    <row r="257" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="258" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A258" s="4"/>
     </row>
@@ -1950,16 +1992,16 @@
     <row r="265" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A265" s="4"/>
     </row>
-    <row r="266" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="266" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A266" s="4"/>
+    </row>
     <row r="267" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A267" s="4"/>
     </row>
     <row r="268" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A268" s="4"/>
     </row>
-    <row r="269" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A269" s="4"/>
-    </row>
+    <row r="269" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="270" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A270" s="4"/>
     </row>
@@ -2056,22 +2098,22 @@
     <row r="301" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A301" s="4"/>
     </row>
+    <row r="302" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A302" s="4"/>
+    </row>
     <row r="303" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A303" s="4"/>
     </row>
     <row r="304" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A304" s="4"/>
     </row>
-    <row r="305" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A305" s="4"/>
-    </row>
     <row r="306" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A306" s="4"/>
     </row>
     <row r="307" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A307" s="4"/>
     </row>
-    <row r="308" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="308" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A308" s="4"/>
     </row>
     <row r="309" spans="1:1" x14ac:dyDescent="0.2">
@@ -2080,7 +2122,7 @@
     <row r="310" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A310" s="4"/>
     </row>
-    <row r="311" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="311" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A311" s="4"/>
     </row>
     <row r="312" spans="1:1" x14ac:dyDescent="0.2">
@@ -2107,8 +2149,8 @@
     <row r="319" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A319" s="4"/>
     </row>
-    <row r="320" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A320" s="7"/>
+    <row r="320" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A320" s="4"/>
     </row>
     <row r="321" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A321" s="4"/>
@@ -2116,8 +2158,8 @@
     <row r="322" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A322" s="4"/>
     </row>
-    <row r="323" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A323" s="4"/>
+    <row r="323" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A323" s="7"/>
     </row>
     <row r="324" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A324" s="4"/>
@@ -2144,7 +2186,7 @@
       <c r="A331" s="4"/>
     </row>
     <row r="332" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A332" s="7"/>
+      <c r="A332" s="4"/>
     </row>
     <row r="333" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A333" s="4"/>
@@ -2153,7 +2195,7 @@
       <c r="A334" s="4"/>
     </row>
     <row r="335" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A335" s="4"/>
+      <c r="A335" s="7"/>
     </row>
     <row r="336" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A336" s="4"/>
@@ -2180,7 +2222,7 @@
       <c r="A343" s="4"/>
     </row>
     <row r="344" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A344" s="7"/>
+      <c r="A344" s="4"/>
     </row>
     <row r="345" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A345" s="4"/>
@@ -2189,7 +2231,7 @@
       <c r="A346" s="4"/>
     </row>
     <row r="347" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A347" s="4"/>
+      <c r="A347" s="7"/>
     </row>
     <row r="348" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A348" s="4"/>
@@ -2215,8 +2257,8 @@
     <row r="355" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A355" s="4"/>
     </row>
-    <row r="356" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A356" s="7"/>
+    <row r="356" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A356" s="4"/>
     </row>
     <row r="357" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A357" s="4"/>
@@ -2224,8 +2266,8 @@
     <row r="358" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A358" s="4"/>
     </row>
-    <row r="359" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A359" s="4"/>
+    <row r="359" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A359" s="7"/>
     </row>
     <row r="360" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A360" s="4"/>
@@ -2251,8 +2293,8 @@
     <row r="367" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A367" s="4"/>
     </row>
-    <row r="368" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A368" s="7"/>
+    <row r="368" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A368" s="4"/>
     </row>
     <row r="369" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A369" s="4"/>
@@ -2260,8 +2302,8 @@
     <row r="370" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A370" s="4"/>
     </row>
-    <row r="371" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A371" s="4"/>
+    <row r="371" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A371" s="7"/>
     </row>
     <row r="372" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A372" s="4"/>
@@ -2288,7 +2330,7 @@
       <c r="A379" s="4"/>
     </row>
     <row r="380" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A380" s="7"/>
+      <c r="A380" s="4"/>
     </row>
     <row r="381" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A381" s="4"/>
@@ -2297,7 +2339,7 @@
       <c r="A382" s="4"/>
     </row>
     <row r="383" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A383" s="4"/>
+      <c r="A383" s="7"/>
     </row>
     <row r="384" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A384" s="4"/>
@@ -2324,7 +2366,7 @@
       <c r="A391" s="4"/>
     </row>
     <row r="392" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A392" s="7"/>
+      <c r="A392" s="4"/>
     </row>
     <row r="393" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A393" s="4"/>
@@ -2333,7 +2375,7 @@
       <c r="A394" s="4"/>
     </row>
     <row r="395" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A395" s="4"/>
+      <c r="A395" s="7"/>
     </row>
     <row r="396" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A396" s="4"/>
@@ -2359,8 +2401,8 @@
     <row r="403" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A403" s="4"/>
     </row>
-    <row r="404" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A404" s="7"/>
+    <row r="404" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A404" s="4"/>
     </row>
     <row r="405" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A405" s="4"/>
@@ -2368,8 +2410,8 @@
     <row r="406" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A406" s="4"/>
     </row>
-    <row r="407" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A407" s="4"/>
+    <row r="407" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A407" s="7"/>
     </row>
     <row r="408" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A408" s="4"/>
@@ -2395,8 +2437,8 @@
     <row r="415" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A415" s="4"/>
     </row>
-    <row r="416" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A416" s="7"/>
+    <row r="416" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A416" s="4"/>
     </row>
     <row r="417" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A417" s="4"/>
@@ -2404,8 +2446,8 @@
     <row r="418" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A418" s="4"/>
     </row>
-    <row r="419" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A419" s="4"/>
+    <row r="419" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A419" s="7"/>
     </row>
     <row r="420" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A420" s="4"/>
@@ -2432,7 +2474,7 @@
       <c r="A427" s="4"/>
     </row>
     <row r="428" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A428" s="7"/>
+      <c r="A428" s="4"/>
     </row>
     <row r="429" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A429" s="4"/>
@@ -2441,7 +2483,7 @@
       <c r="A430" s="4"/>
     </row>
     <row r="431" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A431" s="4"/>
+      <c r="A431" s="7"/>
     </row>
     <row r="432" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A432" s="4"/>
@@ -2468,7 +2510,7 @@
       <c r="A439" s="4"/>
     </row>
     <row r="440" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A440" s="7"/>
+      <c r="A440" s="4"/>
     </row>
     <row r="441" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A441" s="4"/>
@@ -2477,7 +2519,7 @@
       <c r="A442" s="4"/>
     </row>
     <row r="443" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A443" s="4"/>
+      <c r="A443" s="7"/>
     </row>
     <row r="444" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A444" s="4"/>
@@ -2503,22 +2545,22 @@
     <row r="451" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A451" s="4"/>
     </row>
+    <row r="452" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A452" s="4"/>
+    </row>
     <row r="453" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A453" s="4"/>
     </row>
     <row r="454" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A454" s="4"/>
     </row>
-    <row r="455" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A455" s="4"/>
-    </row>
     <row r="456" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A456" s="4"/>
     </row>
     <row r="457" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A457" s="4"/>
     </row>
-    <row r="458" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="458" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A458" s="4"/>
     </row>
     <row r="459" spans="1:1" x14ac:dyDescent="0.2">
@@ -2527,7 +2569,7 @@
     <row r="460" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A460" s="4"/>
     </row>
-    <row r="461" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="461" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A461" s="4"/>
     </row>
     <row r="462" spans="1:1" x14ac:dyDescent="0.2">
@@ -2554,8 +2596,8 @@
     <row r="469" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A469" s="4"/>
     </row>
-    <row r="470" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A470" s="7"/>
+    <row r="470" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A470" s="4"/>
     </row>
     <row r="471" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A471" s="4"/>
@@ -2563,8 +2605,8 @@
     <row r="472" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A472" s="4"/>
     </row>
-    <row r="473" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A473" s="4"/>
+    <row r="473" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A473" s="7"/>
     </row>
     <row r="474" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A474" s="4"/>
@@ -2591,7 +2633,7 @@
       <c r="A481" s="4"/>
     </row>
     <row r="482" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A482" s="7"/>
+      <c r="A482" s="4"/>
     </row>
     <row r="483" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A483" s="4"/>
@@ -2600,7 +2642,7 @@
       <c r="A484" s="4"/>
     </row>
     <row r="485" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A485" s="4"/>
+      <c r="A485" s="7"/>
     </row>
     <row r="486" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A486" s="4"/>
@@ -2627,7 +2669,7 @@
       <c r="A493" s="4"/>
     </row>
     <row r="494" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A494" s="7"/>
+      <c r="A494" s="4"/>
     </row>
     <row r="495" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A495" s="4"/>
@@ -2636,7 +2678,7 @@
       <c r="A496" s="4"/>
     </row>
     <row r="497" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A497" s="4"/>
+      <c r="A497" s="7"/>
     </row>
     <row r="498" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A498" s="4"/>
@@ -2662,8 +2704,8 @@
     <row r="505" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A505" s="4"/>
     </row>
-    <row r="506" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A506" s="7"/>
+    <row r="506" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A506" s="4"/>
     </row>
     <row r="507" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A507" s="4"/>
@@ -2671,8 +2713,8 @@
     <row r="508" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A508" s="4"/>
     </row>
-    <row r="509" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A509" s="4"/>
+    <row r="509" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A509" s="7"/>
     </row>
     <row r="510" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A510" s="4"/>
@@ -2698,8 +2740,8 @@
     <row r="517" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A517" s="4"/>
     </row>
-    <row r="518" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A518" s="7"/>
+    <row r="518" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A518" s="4"/>
     </row>
     <row r="519" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A519" s="4"/>
@@ -2707,8 +2749,8 @@
     <row r="520" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A520" s="4"/>
     </row>
-    <row r="521" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A521" s="4"/>
+    <row r="521" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A521" s="7"/>
     </row>
     <row r="522" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A522" s="4"/>
@@ -2735,7 +2777,7 @@
       <c r="A529" s="4"/>
     </row>
     <row r="530" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A530" s="7"/>
+      <c r="A530" s="4"/>
     </row>
     <row r="531" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A531" s="4"/>
@@ -2744,7 +2786,7 @@
       <c r="A532" s="4"/>
     </row>
     <row r="533" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A533" s="4"/>
+      <c r="A533" s="7"/>
     </row>
     <row r="534" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A534" s="4"/>
@@ -2771,7 +2813,7 @@
       <c r="A541" s="4"/>
     </row>
     <row r="542" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A542" s="7"/>
+      <c r="A542" s="4"/>
     </row>
     <row r="543" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A543" s="4"/>
@@ -2780,7 +2822,7 @@
       <c r="A544" s="4"/>
     </row>
     <row r="545" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A545" s="4"/>
+      <c r="A545" s="7"/>
     </row>
     <row r="546" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A546" s="4"/>
@@ -2806,8 +2848,8 @@
     <row r="553" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A553" s="4"/>
     </row>
-    <row r="554" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A554" s="7"/>
+    <row r="554" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A554" s="4"/>
     </row>
     <row r="555" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A555" s="4"/>
@@ -2815,8 +2857,8 @@
     <row r="556" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A556" s="4"/>
     </row>
-    <row r="557" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A557" s="4"/>
+    <row r="557" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A557" s="7"/>
     </row>
     <row r="558" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A558" s="4"/>
@@ -2842,8 +2884,8 @@
     <row r="565" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A565" s="4"/>
     </row>
-    <row r="566" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A566" s="7"/>
+    <row r="566" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A566" s="4"/>
     </row>
     <row r="567" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A567" s="4"/>
@@ -2851,8 +2893,8 @@
     <row r="568" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A568" s="4"/>
     </row>
-    <row r="569" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A569" s="4"/>
+    <row r="569" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A569" s="7"/>
     </row>
     <row r="570" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A570" s="4"/>
@@ -2879,7 +2921,7 @@
       <c r="A577" s="4"/>
     </row>
     <row r="578" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A578" s="7"/>
+      <c r="A578" s="4"/>
     </row>
     <row r="579" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A579" s="4"/>
@@ -2888,7 +2930,7 @@
       <c r="A580" s="4"/>
     </row>
     <row r="581" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A581" s="4"/>
+      <c r="A581" s="7"/>
     </row>
     <row r="582" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A582" s="4"/>
@@ -2915,7 +2957,7 @@
       <c r="A589" s="4"/>
     </row>
     <row r="590" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A590" s="7"/>
+      <c r="A590" s="4"/>
     </row>
     <row r="591" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A591" s="4"/>
@@ -2924,7 +2966,7 @@
       <c r="A592" s="4"/>
     </row>
     <row r="593" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A593" s="4"/>
+      <c r="A593" s="7"/>
     </row>
     <row r="594" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A594" s="4"/>
@@ -2950,22 +2992,22 @@
     <row r="601" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A601" s="4"/>
     </row>
+    <row r="602" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A602" s="4"/>
+    </row>
     <row r="603" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A603" s="4"/>
     </row>
     <row r="604" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A604" s="4"/>
     </row>
-    <row r="605" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A605" s="4"/>
-    </row>
     <row r="606" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A606" s="4"/>
     </row>
     <row r="607" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A607" s="4"/>
     </row>
-    <row r="608" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="608" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A608" s="4"/>
     </row>
     <row r="609" spans="1:1" x14ac:dyDescent="0.2">
@@ -2974,7 +3016,7 @@
     <row r="610" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A610" s="4"/>
     </row>
-    <row r="611" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="611" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A611" s="4"/>
     </row>
     <row r="612" spans="1:1" x14ac:dyDescent="0.2">
@@ -3001,8 +3043,8 @@
     <row r="619" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A619" s="4"/>
     </row>
-    <row r="620" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A620" s="7"/>
+    <row r="620" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A620" s="4"/>
     </row>
     <row r="621" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A621" s="4"/>
@@ -3010,8 +3052,8 @@
     <row r="622" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A622" s="4"/>
     </row>
-    <row r="623" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A623" s="4"/>
+    <row r="623" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A623" s="7"/>
     </row>
     <row r="624" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A624" s="4"/>
@@ -3038,7 +3080,7 @@
       <c r="A631" s="4"/>
     </row>
     <row r="632" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A632" s="7"/>
+      <c r="A632" s="4"/>
     </row>
     <row r="633" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A633" s="4"/>
@@ -3047,7 +3089,7 @@
       <c r="A634" s="4"/>
     </row>
     <row r="635" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A635" s="4"/>
+      <c r="A635" s="7"/>
     </row>
     <row r="636" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A636" s="4"/>
@@ -3074,7 +3116,7 @@
       <c r="A643" s="4"/>
     </row>
     <row r="644" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A644" s="7"/>
+      <c r="A644" s="4"/>
     </row>
     <row r="645" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A645" s="4"/>
@@ -3083,7 +3125,7 @@
       <c r="A646" s="4"/>
     </row>
     <row r="647" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A647" s="4"/>
+      <c r="A647" s="7"/>
     </row>
     <row r="648" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A648" s="4"/>
@@ -3109,8 +3151,8 @@
     <row r="655" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A655" s="4"/>
     </row>
-    <row r="656" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A656" s="7"/>
+    <row r="656" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A656" s="4"/>
     </row>
     <row r="657" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A657" s="4"/>
@@ -3118,8 +3160,8 @@
     <row r="658" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A658" s="4"/>
     </row>
-    <row r="659" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A659" s="4"/>
+    <row r="659" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A659" s="7"/>
     </row>
     <row r="660" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A660" s="4"/>
@@ -3145,8 +3187,8 @@
     <row r="667" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A667" s="4"/>
     </row>
-    <row r="668" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A668" s="7"/>
+    <row r="668" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A668" s="4"/>
     </row>
     <row r="669" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A669" s="4"/>
@@ -3154,8 +3196,8 @@
     <row r="670" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A670" s="4"/>
     </row>
-    <row r="671" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A671" s="4"/>
+    <row r="671" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A671" s="7"/>
     </row>
     <row r="672" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A672" s="4"/>
@@ -3182,7 +3224,7 @@
       <c r="A679" s="4"/>
     </row>
     <row r="680" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A680" s="7"/>
+      <c r="A680" s="4"/>
     </row>
     <row r="681" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A681" s="4"/>
@@ -3191,7 +3233,7 @@
       <c r="A682" s="4"/>
     </row>
     <row r="683" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A683" s="4"/>
+      <c r="A683" s="7"/>
     </row>
     <row r="684" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A684" s="4"/>
@@ -3218,7 +3260,7 @@
       <c r="A691" s="4"/>
     </row>
     <row r="692" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A692" s="7"/>
+      <c r="A692" s="4"/>
     </row>
     <row r="693" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A693" s="4"/>
@@ -3227,7 +3269,7 @@
       <c r="A694" s="4"/>
     </row>
     <row r="695" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A695" s="4"/>
+      <c r="A695" s="7"/>
     </row>
     <row r="696" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A696" s="4"/>
@@ -3253,8 +3295,8 @@
     <row r="703" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A703" s="4"/>
     </row>
-    <row r="704" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A704" s="7"/>
+    <row r="704" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A704" s="4"/>
     </row>
     <row r="705" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A705" s="4"/>
@@ -3262,8 +3304,8 @@
     <row r="706" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A706" s="4"/>
     </row>
-    <row r="707" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A707" s="4"/>
+    <row r="707" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A707" s="7"/>
     </row>
     <row r="708" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A708" s="4"/>
@@ -3289,8 +3331,8 @@
     <row r="715" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A715" s="4"/>
     </row>
-    <row r="716" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A716" s="7"/>
+    <row r="716" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A716" s="4"/>
     </row>
     <row r="717" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A717" s="4"/>
@@ -3298,8 +3340,8 @@
     <row r="718" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A718" s="4"/>
     </row>
-    <row r="719" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A719" s="4"/>
+    <row r="719" spans="1:1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A719" s="7"/>
     </row>
     <row r="720" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A720" s="4"/>
@@ -3326,7 +3368,7 @@
       <c r="A727" s="4"/>
     </row>
     <row r="728" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A728" s="7"/>
+      <c r="A728" s="4"/>
     </row>
     <row r="729" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A729" s="4"/>
@@ -3335,7 +3377,7 @@
       <c r="A730" s="4"/>
     </row>
     <row r="731" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A731" s="4"/>
+      <c r="A731" s="7"/>
     </row>
     <row r="732" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A732" s="4"/>
@@ -3362,7 +3404,7 @@
       <c r="A739" s="4"/>
     </row>
     <row r="740" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A740" s="7"/>
+      <c r="A740" s="4"/>
     </row>
     <row r="741" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A741" s="4"/>
@@ -3371,7 +3413,7 @@
       <c r="A742" s="4"/>
     </row>
     <row r="743" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A743" s="4"/>
+      <c r="A743" s="7"/>
     </row>
     <row r="744" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A744" s="4"/>
@@ -3396,6 +3438,15 @@
     </row>
     <row r="751" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A751" s="4"/>
+    </row>
+    <row r="752" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A752" s="4"/>
+    </row>
+    <row r="753" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A753" s="4"/>
+    </row>
+    <row r="754" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A754" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>

</xml_diff>